<commit_message>
Cannibalisation summary: one affected URL per row with per-URL role and action
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199Ec3JvGkM5VeF3Edd8KdB
</commit_message>
<xml_diff>
--- a/Solent-Power-Client-Presentation-Workbook.xlsx
+++ b/Solent-Power-Client-Presentation-Workbook.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Keyword Universe'!$A$1:$H$196</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Keyword-Page Map'!$A$1:$J$156</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Cannibalisation Summary'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Cannibalisation Summary'!$A$1:$E$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Redirects &amp; New Titles'!$A$1:$F$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Internal Links - Commercial'!$A$1:$D$236</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Internal Links - Blog'!$A$1:$D$191</definedName>
@@ -13224,13 +13224,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13246,12 +13247,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Pages involved</t>
+          <t>Affected URL</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>What to do</t>
+          <t>Role today</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
         </is>
       </c>
     </row>
@@ -13263,220 +13269,937 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>One buying intent (servicing/maintenance/contracts) spread over SIX pages. Google shows a different Solent page depending on the query — none of them well. 60,559 impressions in 90 days produced 27 clicks.</t>
+          <t>One buying intent (servicing / maintenance / contracts) spread over six pages — Google shows a different Solent page depending on the query, none of them well. 60,559 impressions in 90 days → 27 clicks.</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>/generator-service-maintenance/ (the rightful owner) · /how-often-should-generators-be-serviced/ (blog — currently WINS 'servicing and maintenance') · /knowledge-base/ (wins 'diesel generator maintenance') · /locations/surrey/ (wins 'generator service') · /hampshire-generators/ (wins 'repair near me') · /diesel-generator-service-contracts-uk-2026/</t>
+          <t>/generator-service-maintenance/</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>KEEP ALL PAGES — retitle so only the service page carries commercial servicing terms; blog keeps 'how often', locations keep '{service} {place}'. No redirects needed in this group.</t>
+          <t>The rightful owner — currently loses to the pages below</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>KEEP + REBUILD as the only page titled for servicing/maintenance/contracts terms (P1)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>2 · UPS — two live trees</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>The UPS migration is HALF-DONE: /ups/* and /uninterruptible-power-supplies/* are both live with identical titles ('3 Phase UPS' twice, 'Modular UPS Systems' twice). The site competes with itself on every UPS category today.</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>/ups/three-phase/ vs /uninterruptible-power-supplies/three-phase-ups/ · /ups/modular/ vs …/modular/ · /ups/tower/ vs …/tower/ · /ups/configurable-output/ vs …/configurable-output/ · /ups/single-phase/ (new-tree home MISSING) · /ups/rack-mount/</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>MERGE: 301 every old /ups/* URL to its new-tree twin; create /uninterruptible-power-supplies/single-phase-ups/ first. Then write unique descriptions (audit flags duplicates across UPS children).</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1 · Servicing &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>/how-often-should-generators-be-serviced/</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Blog post — currently WINS 'generator servicing and maintenance'</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>RETITLE to the question ('How often should a generator be serviced?'); link down to the service page with exact anchor</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>3 · kVA vs kW size series</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Two parallel size ladders (19 kVA + 21 kW pages) chase the same buyers. Google sometimes ranks the 25kVA page for '25kw generator' and vice versa. And 200kVA ≠ 200kW, so same-number pages actively mislead.</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>/generators/{N}kva/ ×19 live · /generators/{N}kw/ ×21 live</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>MERGE (agreed): every kW page 301s ONCE to the kVA page covering its converted rating (kW÷0.8, round up). Full mapping + new titles/H1s on the Redirects tab. kW number goes into the kVA titles BEFORE redirecting.</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1 · Servicing &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>/knowledge-base/</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Hub page — currently wins 'diesel generator maintenance'</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Remove commercial servicing terms from title; becomes a pure guide index</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4 · Products beating their own categories</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>For '30kva generator', '250 kva generator' etc., a single PRODUCT page outranks the category that should win — validated against the live SERPs, where competitors rank size CATEGORY pages.</t>
-        </is>
-      </c>
+          <t>1 · Servicing &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>e.g. /product/…/cps-ap30s-30kva…/ outranks /generators/30kva/ · same at 45/60/80/250/300kVA</t>
+          <t>/locations/surrey/</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>RETITLE products to their model terms ('CPS AP30S 30kVA Diesel Generator'); each product exact-anchor links UP to its size category. Categories get the merchandised titles (Redirects tab pattern).</t>
+          <t>Location page — currently wins national 'generator service'</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>RETITLE to 'Generator Servicing &amp; Repair in Surrey' — geo terms only</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>5 · 'Commercial generator' — three owners</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Three different pages rank for 'commercial generator' depending on the day, including the hospital page.</t>
-        </is>
-      </c>
+          <t>1 · Servicing &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>/generators/industrial-generators/ · /hospital-generators/ · /generator-sales/emergency-generator-sales/</t>
+          <t>/hampshire-generators/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>/generators/industrial-generators/ owns industrial + commercial (title covers both). Hospital page retitles to healthcare terms only.</t>
+          <t>Local hub — wins 'generator repair near me' family</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>KEEP those local/near-me terms — this page is doing its job; just stop it titling national terms</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>6 · Brand pages — three URL patterns</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Most brands exist as a shop taxonomy page (/brand/), a content page (/brands/), and sometimes a sales page — splitting the brand's authority 2-3 ways. Three /brand/ pages are now 404 (teksan, cps, evopower).</t>
-        </is>
-      </c>
+          <t>1 · Servicing &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>/brand/{x}/ ×7 · /brands/{x}/ ×10 · /generator-sales/hyundai-generators/ etc. · 404s: /brand/teksan/, /brand/cps/, /brand/evopower/</t>
+          <t>/diesel-generator-service-contracts-uk-2026/</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ONE page per brand at /brands/{x}/. 301 the /brand/ taxonomy + sales duplicates in; fix the three 404s (301 to /brands/ twin or products).</t>
+          <t>New article overlapping the contracts intent</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Feed it: link prominently to the service page; don't let it title 'service contracts' commercially</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>7 · Sizing &amp; kVA guides</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Two sizing guides + a kVA-vs-kW explainer split the 'what size generator' demand; none rank top 3.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>/generator-sizing-specification/ · /what-size-generator-do-i-need/ · /the-differences-between-kva-and-kw/</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>MERGE the two sizing guides (301 what-size into sizing-specification). Keep kVA-vs-kW separate (different question) but rebuild with the conversion chart and links to every size page.</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>The UPS migration is half-done: old and new category trees are BOTH live with identical titles. The site competes with itself on every UPS term today.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>/uninterruptible-power-supplies/</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>New hub — the keeper</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>KEEP — becomes the UPS hub; write unique descriptions for children</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>8 · Fuel services</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Fuel intent spread across two service pages, a blog and two hardware categories; 'fuel polishing' (300/mo, zero competition) has no owner.</t>
-        </is>
-      </c>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>/generator-fuel-services/ · /fuel-sampling-and-testing-services/ · /generator-fuel-types/ (blog) · /fuel-storage-tanks/ · /fuel-bowser/</t>
+          <t>/ups/three-phase/</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>/generator-fuel-services/ becomes the fuel hub with a fuel-polishing section (own child page later); sampling/testing stays but cross-linked as part of one offer; hardware categories unchanged.</t>
+          <t>Old twin of /uninterruptible-power-supplies/three-phase-ups/ (identical title '3 Phase UPS')</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>301 → /uninterruptible-power-supplies/three-phase-ups/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>9 · Contingency planning — new duplication</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>A new page shipped recently overlaps the existing contingency page — watch this doesn't become servicing 2.0.</t>
-        </is>
-      </c>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>/contingency-power-plan/ · /power-contingency-planning-30-days-uk/ (new)</t>
+          <t>/ups/modular/</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Differentiate now: contingency-power-plan = the service page; 30-days page = the campaign/guide, retitled and linking to it (or merge if content is 80% same).</t>
+          <t>Old twin — identical title 'Modular UPS Systems'</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>301 → /uninterruptible-power-supplies/modular/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>/ups/tower/</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Old twin — identical title 'Tower UPS'</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>301 → /uninterruptible-power-supplies/tower/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>/ups/configurable-output/</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Old twin</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>301 → /uninterruptible-power-supplies/configurable-output/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>/ups/single-phase/</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Old page whose new-tree home DOESN'T EXIST yet</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>CREATE /uninterruptible-power-supplies/single-phase-ups/ first, then 301 this into it</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>/ups/rack-mount/</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Old page, no new-tree twin</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>CREATE or fold into the hub as a section, then 301</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2 · UPS — two live trees</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>/what-is-an-uninterruptible-power-supply/</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Blog — the site's best-ranking UPS URL today (pos 26-40)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Keeps the 'what is' question; links down to the hub with commercial anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>3 · kVA vs kW size series</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Two parallel size ladders (19 kVA + 21 kW pages) chase the same buyers, and 200kVA ≠ 200kW so same-number comparisons actively mislead. Client-agreed fix: one kVA-only ladder.</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>/generators/{N}kva/ — 19 live pages</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>The keepers</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Each gets the new title/H1 with its kW equivalent (see Redirects tab) BEFORE the kW redirects fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>3 · kVA vs kW size series</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>/generators/{N}kw/ — 21 live pages</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>The duplicates</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Each 301s ONCE to the kVA page covering its converted rating (kW ÷ 0.8, rounded up) — full per-page mapping on the Redirects tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>3 · kVA vs kW size series</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>/generators/1250kva/</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>404 right now (the live page is /generators/1250-kva/)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>301 the 404 to the hyphenated page immediately</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>4 · Products beating their own categories</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>For size searches like '30kva generator', a single product page outranks the category that should win — competitors win these SERPs with category pages.</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>/generators/30kva/</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Category — should own '30kva generator' but doesn't rank</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Merchandised title + intro; gains exact-anchor links from its products</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>4 · Products beating their own categories</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>/product/diesel-generators/cps-ap30s-30kva-diesel-generator/</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Product — currently ranks pos 7 for the size term</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>RETITLE to model term 'CPS AP30S 30kVA Diesel Generator'; link up to /generators/30kva/ with anchor '30kVA generators'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>4 · Products beating their own categories</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>(same pattern at 45 / 60 / 80 / 250 / 300kVA)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Product outranks or replaces category</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Same fix: product → model term, category → size term, exact-anchor link up</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>5 · 'Commercial generator' — three owners</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Three different pages rank for 'commercial generator' depending on the day, including the hospital page.</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>/generators/industrial-generators/</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Ranks pos 3-7 for industrial + commercial terms</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>THE owner — title covers 'Industrial &amp; Commercial Generators'</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>5 · 'Commercial generator' — three owners</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>/hospital-generators/</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Currently pos 1 for 'commercial generator' (wrong job)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>RETITLE to healthcare terms only ('Hospital &amp; Healthcare Generators — HTM 06-01')</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>5 · 'Commercial generator' — three owners</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>/generator-sales/emergency-generator-sales/</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Also ranks for commercial/emergency generator</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Keeps 'emergency generator' (purchase intent) only</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>6 · Brand pages — three URL patterns</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Most brands exist as a shop taxonomy page (/brand/), a content page (/brands/), and sometimes a sales page — splitting each brand's authority 2-3 ways. Three /brand/ pages are now 404.</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>/brands/{brand}/ — 10 pages</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>The keepers (content + service pages)</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Canonical pattern: one page per brand, sales + servicing together, dealer status in title</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>6 · Brand pages — three URL patterns</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>/brand/himoinsa/ · /brand/cat/ · /brand/pramac/ etc. (7 live)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Woo taxonomy duplicates</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>301 each into its /brands/ twin (or its category if no twin exists)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>6 · Brand pages — three URL patterns</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>/brand/teksan/ · /brand/cps/ · /brand/evopower/</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>404 right now</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>301 to the matching /brands/ page or the brand's product listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>6 · Brand pages — three URL patterns</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>/generator-sales/hyundai-generators/ · /generator-sales/teksan-generators/</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Third pattern — sales duplicates</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>301 into the /brands/ twin</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>6 · Brand pages — three URL patterns</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>/brand/hyundai/</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Currently noindexed (half-fix)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Replace noindex with a 301 when consolidation ships</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>7 · Sizing &amp; kVA guides</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Two sizing guides + a kVA-vs-kW explainer split the 'what size generator' demand; none rank top 3.</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>/generator-sizing-specification/</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>The keeper</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Absorbs the other guide; hosts the size chart; links to every size page (the ladder's link engine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>7 · Sizing &amp; kVA guides</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>/what-size-generator-do-i-need/</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate sizing guide</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>301 → /generator-sizing-specification/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>7 · Sizing &amp; kVA guides</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>/the-differences-between-kva-and-kw/</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Separate question — keep</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>REBUILD with conversion chart (currently pos 34 for 'kva'); links to size ladder</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>8 · Fuel services</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Fuel intent spread across two service pages, a blog and hardware categories; 'fuel polishing' (300/mo, zero competition) has no owner.</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>/generator-fuel-services/</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>The keeper — becomes the fuel hub</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Add fuel polishing section (own child later) — 300/mo at KD 0 unowned</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>8 · Fuel services</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>/fuel-sampling-and-testing-services/</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Overlapping service page</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>KEEP but position as part of one fuel offer; heavy cross-links both ways</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>8 · Fuel services</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>/generator-fuel-types/</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Keeps informational fuel terms; links down to fuel services</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>8 · Fuel services</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>/fuel-storage-tanks/ · /fuel-bowser/ · /fuel-pods/</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Hardware categories</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Unchanged — link from the fuel hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>9 · Contingency planning — new duplication</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>A newly shipped page overlaps the existing contingency page — catch it before it becomes servicing 2.0.</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>/contingency-power-plan/</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Existing service page</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>THE owner of contingency/continuity planning terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>9 · Contingency planning — new duplication</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>/power-contingency-planning-30-days-uk/</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>New page (shipped recently)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Position as the campaign/guide ('30-day plan') linking to the service page — or merge if 80% same content</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
           <t>10 · BESS</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Two battery storage pages, one intent.</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>/battery-energy-storage-solutions-bess/ · /battery-energy-storage-systems/</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Merge to one (keep the stronger URL, 301 the other). Low priority — the only high-difficulty cluster (KD 43).</t>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Two battery storage pages, one intent. Only high-difficulty cluster in the plan (KD 43) — low priority.</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>/battery-energy-storage-solutions-bess/</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Product category version</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Pick the stronger of the two as keeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>10 · BESS</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>/battery-energy-storage-systems/</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Service page version</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>301 the weaker into the keeper</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D11"/>
+  <autoFilter ref="A1:E40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>